<commit_message>
Update SpringSmash 2026 budget with final planning costs and leaderboard UI
- Updated Operations: waterslide $1,999, Rugged Warrior $1,799, Dunk Tank $449, Wrecking Ball $599, generators $189/unit, snowcone machines $125/unit, snowcone servings $0.70/unit, Freezies $300 bulk
- Added new Operations line items: Slip and Slide ($399) and Rain Day Fee ($900)
- Added Marketing: T-Shirts ($3,600) under Merchandise/Swag
- Added springsmash donation leaderboard App.tsx and index.css

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/KinetIQ_Projected_Cash_Flow_updated.xlsx
+++ b/KinetIQ_Projected_Cash_Flow_updated.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://standrewsaurora-my.sharepoint.com/personal/jayden_leung_sac_on_ca/Documents/Desktop/12-02 School Folder/McEwen Business Leadership/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="11_D0D3B489D174F4DF643C0817485DCE3A87C54A00" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{279A7848-A46F-4B0F-B1FB-9D7170320D09}"/>
+  <xr:revisionPtr revIDLastSave="124" documentId="11_D0D3B489D174F4DF643C0817485DCE3A87C54A00" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3B734F7-3339-4B34-9B3B-D7FEF8AC8747}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="67">
   <si>
     <t>KinetIQ Projected Cash Flow Statement</t>
   </si>
@@ -62,9 +62,6 @@
     <t>Cash In</t>
   </si>
   <si>
-    <t>Estimated revenue</t>
-  </si>
-  <si>
     <t>Cash Out</t>
   </si>
   <si>
@@ -230,7 +227,64 @@
     <t>Yearly Deficit</t>
   </si>
   <si>
-    <t>Cumulative</t>
+    <r>
+      <t xml:space="preserve">Estimated revenue </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(UPSIDE CASE)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Estimated revenue </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(BASE CASE)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Cumulative </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(BASE CASE)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Cumulative </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>(UPSIDE CASE)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -241,7 +295,7 @@
     <numFmt numFmtId="164" formatCode="\$#,##0"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -268,6 +322,26 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -342,7 +416,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -360,6 +434,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -662,7 +737,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G65"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -714,78 +789,78 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="B4" s="4">
         <v>446785</v>
       </c>
       <c r="C4" s="4">
-        <v>682249</v>
+        <v>558481</v>
       </c>
       <c r="D4" s="4">
-        <v>826580</v>
+        <v>698101</v>
       </c>
       <c r="E4" s="4">
-        <v>1157511</v>
+        <v>872626</v>
       </c>
       <c r="F4" s="4">
-        <v>1462389</v>
+        <v>1090783</v>
       </c>
       <c r="G4" s="9">
         <f>SUM(B4:F4)</f>
-        <v>4575514</v>
+        <v>3666776</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="3"/>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="A5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="4">
+        <v>446785</v>
+      </c>
+      <c r="C5" s="4">
+        <v>580821</v>
+      </c>
+      <c r="D5" s="4">
+        <v>755067</v>
+      </c>
+      <c r="E5" s="4">
+        <v>981587</v>
+      </c>
+      <c r="F5" s="4">
+        <v>1276063</v>
+      </c>
+      <c r="G5" s="9">
+        <f>SUM(B5:F5)</f>
+        <v>4040323</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="A6" s="3"/>
       <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
+      <c r="C6" s="4"/>
+      <c r="D6" s="4"/>
+      <c r="E6" s="4"/>
+      <c r="F6" s="4"/>
       <c r="G6" s="3"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="5">
-        <v>15000</v>
-      </c>
-      <c r="C7" s="5">
-        <v>0</v>
-      </c>
-      <c r="D7" s="5">
-        <v>0</v>
-      </c>
-      <c r="E7" s="5">
-        <v>0</v>
-      </c>
-      <c r="F7" s="5">
-        <v>0</v>
-      </c>
-      <c r="G7" s="5">
-        <f>SUM(B7:F7)</f>
-        <v>15000</v>
-      </c>
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B8" s="5">
-        <v>134</v>
+        <v>15000</v>
       </c>
       <c r="C8" s="5">
         <v>0</v>
@@ -800,16 +875,16 @@
         <v>0</v>
       </c>
       <c r="G8" s="5">
-        <f t="shared" ref="G8:G58" si="0">SUM(B8:F8)</f>
-        <v>134</v>
+        <f>SUM(B8:F8)</f>
+        <v>15000</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B9" s="5">
-        <v>21600</v>
+        <v>134</v>
       </c>
       <c r="C9" s="5">
         <v>0</v>
@@ -824,16 +899,16 @@
         <v>0</v>
       </c>
       <c r="G9" s="5">
-        <f t="shared" si="0"/>
-        <v>21600</v>
+        <f t="shared" ref="G9:G59" si="0">SUM(B9:F9)</f>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B10" s="5">
-        <v>49950</v>
+        <v>21600</v>
       </c>
       <c r="C10" s="5">
         <v>0</v>
@@ -849,15 +924,15 @@
       </c>
       <c r="G10" s="5">
         <f t="shared" si="0"/>
-        <v>49950</v>
+        <v>21600</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B11" s="5">
-        <v>30000</v>
+        <v>49950</v>
       </c>
       <c r="C11" s="5">
         <v>0</v>
@@ -873,15 +948,15 @@
       </c>
       <c r="G11" s="5">
         <f t="shared" si="0"/>
-        <v>30000</v>
+        <v>49950</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B12" s="5">
-        <v>2000</v>
+        <v>30000</v>
       </c>
       <c r="C12" s="5">
         <v>0</v>
@@ -897,15 +972,15 @@
       </c>
       <c r="G12" s="5">
         <f t="shared" si="0"/>
-        <v>2000</v>
+        <v>30000</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B13" s="5">
-        <v>1740</v>
+        <v>2000</v>
       </c>
       <c r="C13" s="5">
         <v>0</v>
@@ -921,15 +996,15 @@
       </c>
       <c r="G13" s="5">
         <f t="shared" si="0"/>
-        <v>1740</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B14" s="5">
-        <v>20000</v>
+        <v>1740</v>
       </c>
       <c r="C14" s="5">
         <v>0</v>
@@ -945,15 +1020,15 @@
       </c>
       <c r="G14" s="5">
         <f t="shared" si="0"/>
-        <v>20000</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B15" s="5">
-        <v>21600</v>
+        <v>20000</v>
       </c>
       <c r="C15" s="5">
         <v>0</v>
@@ -969,15 +1044,15 @@
       </c>
       <c r="G15" s="5">
         <f t="shared" si="0"/>
-        <v>21600</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B16" s="5">
-        <v>10000</v>
+        <v>21600</v>
       </c>
       <c r="C16" s="5">
         <v>0</v>
@@ -993,15 +1068,15 @@
       </c>
       <c r="G16" s="5">
         <f t="shared" si="0"/>
-        <v>10000</v>
+        <v>21600</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B17" s="5">
-        <v>25000</v>
+        <v>10000</v>
       </c>
       <c r="C17" s="5">
         <v>0</v>
@@ -1017,15 +1092,15 @@
       </c>
       <c r="G17" s="5">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B18" s="5">
-        <v>8325</v>
+        <v>25000</v>
       </c>
       <c r="C18" s="5">
         <v>0</v>
@@ -1041,15 +1116,15 @@
       </c>
       <c r="G18" s="5">
         <f t="shared" si="0"/>
-        <v>8325</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B19" s="5">
-        <v>330</v>
+        <v>8325</v>
       </c>
       <c r="C19" s="5">
         <v>0</v>
@@ -1065,15 +1140,15 @@
       </c>
       <c r="G19" s="5">
         <f t="shared" si="0"/>
-        <v>330</v>
+        <v>8325</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B20" s="5">
-        <v>5000</v>
+        <v>330</v>
       </c>
       <c r="C20" s="5">
         <v>0</v>
@@ -1089,1049 +1164,1102 @@
       </c>
       <c r="G20" s="5">
         <f t="shared" si="0"/>
-        <v>5000</v>
+        <v>330</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B21" s="5">
-        <v>2000</v>
+        <v>5000</v>
       </c>
       <c r="C21" s="5">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="D21" s="5">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="E21" s="5">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="F21" s="5">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="G21" s="5">
         <f t="shared" si="0"/>
-        <v>10000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B22" s="5">
-        <v>900</v>
+        <v>2000</v>
       </c>
       <c r="C22" s="5">
-        <v>900</v>
+        <v>2000</v>
       </c>
       <c r="D22" s="5">
-        <v>900</v>
+        <v>2000</v>
       </c>
       <c r="E22" s="5">
-        <v>900</v>
+        <v>2000</v>
       </c>
       <c r="F22" s="5">
-        <v>900</v>
+        <v>2000</v>
       </c>
       <c r="G22" s="5">
         <f t="shared" si="0"/>
-        <v>4500</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B23" s="5">
-        <v>90000</v>
+        <v>900</v>
       </c>
       <c r="C23" s="5">
-        <v>90000</v>
+        <v>900</v>
       </c>
       <c r="D23" s="5">
-        <v>90000</v>
+        <v>900</v>
       </c>
       <c r="E23" s="5">
-        <v>90000</v>
+        <v>900</v>
       </c>
       <c r="F23" s="5">
-        <v>90000</v>
+        <v>900</v>
       </c>
       <c r="G23" s="5">
         <f t="shared" si="0"/>
-        <v>450000</v>
+        <v>4500</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B24" s="5">
-        <v>80000</v>
+        <v>90000</v>
       </c>
       <c r="C24" s="5">
-        <v>80000</v>
+        <v>90000</v>
       </c>
       <c r="D24" s="5">
-        <v>80000</v>
+        <v>90000</v>
       </c>
       <c r="E24" s="5">
-        <v>80000</v>
+        <v>90000</v>
       </c>
       <c r="F24" s="5">
-        <v>80000</v>
+        <v>90000</v>
       </c>
       <c r="G24" s="5">
         <f t="shared" si="0"/>
-        <v>400000</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B25" s="5">
-        <v>7500</v>
+        <v>80000</v>
       </c>
       <c r="C25" s="5">
-        <v>7500</v>
+        <v>80000</v>
       </c>
       <c r="D25" s="5">
-        <v>7500</v>
+        <v>80000</v>
       </c>
       <c r="E25" s="5">
-        <v>7500</v>
+        <v>80000</v>
       </c>
       <c r="F25" s="5">
-        <v>7500</v>
+        <v>80000</v>
       </c>
       <c r="G25" s="5">
         <f t="shared" si="0"/>
-        <v>37500</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B26" s="5">
-        <v>99</v>
+        <v>7500</v>
       </c>
       <c r="C26" s="5">
-        <v>99</v>
+        <v>7500</v>
       </c>
       <c r="D26" s="5">
-        <v>99</v>
+        <v>7500</v>
       </c>
       <c r="E26" s="5">
-        <v>99</v>
+        <v>7500</v>
       </c>
       <c r="F26" s="5">
-        <v>99</v>
+        <v>7500</v>
       </c>
       <c r="G26" s="5">
         <f t="shared" si="0"/>
-        <v>495</v>
+        <v>37500</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B27" s="5">
-        <v>800</v>
+        <v>99</v>
       </c>
       <c r="C27" s="5">
-        <v>800</v>
+        <v>99</v>
       </c>
       <c r="D27" s="5">
-        <v>800</v>
+        <v>99</v>
       </c>
       <c r="E27" s="5">
-        <v>800</v>
+        <v>99</v>
       </c>
       <c r="F27" s="5">
-        <v>800</v>
+        <v>99</v>
       </c>
       <c r="G27" s="5">
         <f t="shared" si="0"/>
-        <v>4000</v>
+        <v>495</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B28" s="5">
-        <v>360</v>
+        <v>800</v>
       </c>
       <c r="C28" s="5">
-        <v>360</v>
+        <v>800</v>
       </c>
       <c r="D28" s="5">
-        <v>360</v>
+        <v>800</v>
       </c>
       <c r="E28" s="5">
-        <v>360</v>
+        <v>800</v>
       </c>
       <c r="F28" s="5">
-        <v>360</v>
+        <v>800</v>
       </c>
       <c r="G28" s="5">
         <f t="shared" si="0"/>
-        <v>1800</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B29" s="5">
-        <v>540</v>
+        <v>360</v>
       </c>
       <c r="C29" s="5">
-        <v>540</v>
+        <v>360</v>
       </c>
       <c r="D29" s="5">
-        <v>540</v>
+        <v>360</v>
       </c>
       <c r="E29" s="5">
-        <v>540</v>
+        <v>360</v>
       </c>
       <c r="F29" s="5">
-        <v>540</v>
+        <v>360</v>
       </c>
       <c r="G29" s="5">
         <f t="shared" si="0"/>
-        <v>2700</v>
+        <v>1800</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B30" s="5">
-        <v>300</v>
+        <v>540</v>
       </c>
       <c r="C30" s="5">
-        <v>300</v>
+        <v>540</v>
       </c>
       <c r="D30" s="5">
-        <v>300</v>
+        <v>540</v>
       </c>
       <c r="E30" s="5">
-        <v>300</v>
+        <v>540</v>
       </c>
       <c r="F30" s="5">
-        <v>300</v>
+        <v>540</v>
       </c>
       <c r="G30" s="5">
         <f t="shared" si="0"/>
-        <v>1500</v>
+        <v>2700</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B31" s="5">
-        <v>4000</v>
+        <v>300</v>
       </c>
       <c r="C31" s="5">
-        <v>4000</v>
+        <v>300</v>
       </c>
       <c r="D31" s="5">
-        <v>4000</v>
+        <v>300</v>
       </c>
       <c r="E31" s="5">
-        <v>4000</v>
+        <v>300</v>
       </c>
       <c r="F31" s="5">
-        <v>4000</v>
+        <v>300</v>
       </c>
       <c r="G31" s="5">
         <f t="shared" si="0"/>
-        <v>20000</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B32" s="5">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="C32" s="5">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="D32" s="5">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="E32" s="5">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="F32" s="5">
-        <v>10000</v>
+        <v>4000</v>
       </c>
       <c r="G32" s="5">
         <f t="shared" si="0"/>
-        <v>50000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B33" s="5">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="C33" s="5">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="D33" s="5">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="E33" s="5">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="F33" s="5">
-        <v>30000</v>
+        <v>10000</v>
       </c>
       <c r="G33" s="5">
         <f t="shared" si="0"/>
-        <v>150000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B34" s="5">
-        <v>696</v>
+        <v>30000</v>
       </c>
       <c r="C34" s="5">
-        <v>696</v>
+        <v>30000</v>
       </c>
       <c r="D34" s="5">
-        <v>696</v>
+        <v>30000</v>
       </c>
       <c r="E34" s="5">
-        <v>696</v>
+        <v>30000</v>
       </c>
       <c r="F34" s="5">
-        <v>696</v>
+        <v>30000</v>
       </c>
       <c r="G34" s="5">
         <f t="shared" si="0"/>
-        <v>3480</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B35" s="5">
-        <v>66000</v>
+        <v>696</v>
       </c>
       <c r="C35" s="5">
-        <v>66000</v>
+        <v>696</v>
       </c>
       <c r="D35" s="5">
-        <v>66000</v>
+        <v>696</v>
       </c>
       <c r="E35" s="5">
-        <v>66000</v>
+        <v>696</v>
       </c>
       <c r="F35" s="5">
-        <v>66000</v>
+        <v>696</v>
       </c>
       <c r="G35" s="5">
         <f t="shared" si="0"/>
-        <v>330000</v>
+        <v>3480</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B36" s="5">
-        <v>20</v>
+        <v>66000</v>
       </c>
       <c r="C36" s="5">
-        <v>20</v>
+        <v>66000</v>
       </c>
       <c r="D36" s="5">
-        <v>20</v>
+        <v>66000</v>
       </c>
       <c r="E36" s="5">
-        <v>20</v>
+        <v>66000</v>
       </c>
       <c r="F36" s="5">
-        <v>20</v>
+        <v>66000</v>
       </c>
       <c r="G36" s="5">
         <f t="shared" si="0"/>
-        <v>100</v>
+        <v>330000</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B37" s="5">
-        <v>288</v>
+        <v>20</v>
       </c>
       <c r="C37" s="5">
-        <v>288</v>
+        <v>20</v>
       </c>
       <c r="D37" s="5">
-        <v>288</v>
+        <v>20</v>
       </c>
       <c r="E37" s="5">
-        <v>288</v>
+        <v>20</v>
       </c>
       <c r="F37" s="5">
-        <v>288</v>
+        <v>20</v>
       </c>
       <c r="G37" s="5">
         <f t="shared" si="0"/>
-        <v>1440</v>
+        <v>100</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B38" s="5">
-        <v>450</v>
+        <v>288</v>
       </c>
       <c r="C38" s="5">
-        <v>450</v>
+        <v>288</v>
       </c>
       <c r="D38" s="5">
-        <v>450</v>
+        <v>288</v>
       </c>
       <c r="E38" s="5">
-        <v>450</v>
+        <v>288</v>
       </c>
       <c r="F38" s="5">
-        <v>450</v>
+        <v>288</v>
       </c>
       <c r="G38" s="5">
         <f t="shared" si="0"/>
-        <v>2250</v>
+        <v>1440</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B39" s="5">
-        <v>10200</v>
+        <v>450</v>
       </c>
       <c r="C39" s="5">
-        <v>10200</v>
+        <v>450</v>
       </c>
       <c r="D39" s="5">
-        <v>10200</v>
+        <v>450</v>
       </c>
       <c r="E39" s="5">
-        <v>10200</v>
+        <v>450</v>
       </c>
       <c r="F39" s="5">
-        <v>10200</v>
+        <v>450</v>
       </c>
       <c r="G39" s="5">
         <f t="shared" si="0"/>
-        <v>51000</v>
+        <v>2250</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B40" s="5">
-        <v>1626</v>
+        <v>10200</v>
       </c>
       <c r="C40" s="5">
-        <v>1626</v>
+        <v>10200</v>
       </c>
       <c r="D40" s="5">
-        <v>1626</v>
+        <v>10200</v>
       </c>
       <c r="E40" s="5">
-        <v>1626</v>
+        <v>10200</v>
       </c>
       <c r="F40" s="5">
-        <v>1626</v>
+        <v>10200</v>
       </c>
       <c r="G40" s="5">
         <f t="shared" si="0"/>
-        <v>8130</v>
+        <v>51000</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B41" s="5">
-        <v>23000</v>
+        <v>1626</v>
       </c>
       <c r="C41" s="5">
-        <v>23000</v>
+        <v>1626</v>
       </c>
       <c r="D41" s="5">
-        <v>23000</v>
+        <v>1626</v>
       </c>
       <c r="E41" s="5">
-        <v>23000</v>
+        <v>1626</v>
       </c>
       <c r="F41" s="5">
-        <v>23000</v>
+        <v>1626</v>
       </c>
       <c r="G41" s="5">
         <f t="shared" si="0"/>
-        <v>115000</v>
+        <v>8130</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B42" s="5">
-        <v>2400</v>
+        <v>23000</v>
       </c>
       <c r="C42" s="5">
-        <v>2400</v>
+        <v>23000</v>
       </c>
       <c r="D42" s="5">
-        <v>2400</v>
+        <v>23000</v>
       </c>
       <c r="E42" s="5">
-        <v>2400</v>
+        <v>23000</v>
       </c>
       <c r="F42" s="5">
-        <v>2400</v>
+        <v>23000</v>
       </c>
       <c r="G42" s="5">
         <f t="shared" si="0"/>
-        <v>12000</v>
+        <v>115000</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B43" s="5">
-        <v>19584</v>
+        <v>2400</v>
       </c>
       <c r="C43" s="5">
-        <v>19584</v>
+        <v>2400</v>
       </c>
       <c r="D43" s="5">
-        <v>19584</v>
+        <v>2400</v>
       </c>
       <c r="E43" s="5">
-        <v>19584</v>
+        <v>2400</v>
       </c>
       <c r="F43" s="5">
-        <v>19584</v>
+        <v>2400</v>
       </c>
       <c r="G43" s="5">
         <f t="shared" si="0"/>
-        <v>97920</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B44" s="5">
-        <v>2500</v>
+        <v>19584</v>
       </c>
       <c r="C44" s="5">
-        <v>2500</v>
+        <v>19584</v>
       </c>
       <c r="D44" s="5">
-        <v>2500</v>
+        <v>19584</v>
       </c>
       <c r="E44" s="5">
-        <v>2500</v>
+        <v>19584</v>
       </c>
       <c r="F44" s="5">
-        <v>2500</v>
+        <v>19584</v>
       </c>
       <c r="G44" s="5">
         <f t="shared" si="0"/>
-        <v>12500</v>
+        <v>97920</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B45" s="5">
-        <v>12000</v>
+        <v>2500</v>
       </c>
       <c r="C45" s="5">
-        <v>12000</v>
+        <v>2500</v>
       </c>
       <c r="D45" s="5">
-        <v>12000</v>
+        <v>2500</v>
       </c>
       <c r="E45" s="5">
-        <v>12000</v>
+        <v>2500</v>
       </c>
       <c r="F45" s="5">
-        <v>12000</v>
+        <v>2500</v>
       </c>
       <c r="G45" s="5">
         <f t="shared" si="0"/>
-        <v>60000</v>
+        <v>12500</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B46" s="5">
-        <v>10419.959999999999</v>
+        <v>12000</v>
       </c>
       <c r="C46" s="5">
-        <v>10419.959999999999</v>
+        <v>12000</v>
       </c>
       <c r="D46" s="5">
-        <v>10419.959999999999</v>
+        <v>12000</v>
       </c>
       <c r="E46" s="5">
-        <v>10419.959999999999</v>
+        <v>12000</v>
       </c>
       <c r="F46" s="5">
-        <v>10419.959999999999</v>
+        <v>12000</v>
       </c>
       <c r="G46" s="5">
         <f t="shared" si="0"/>
-        <v>52099.799999999996</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B47" s="5">
-        <v>1000</v>
+        <v>10419.959999999999</v>
       </c>
       <c r="C47" s="5">
-        <v>1000</v>
+        <v>10419.959999999999</v>
       </c>
       <c r="D47" s="5">
-        <v>1000</v>
+        <v>10419.959999999999</v>
       </c>
       <c r="E47" s="5">
-        <v>1000</v>
+        <v>10419.959999999999</v>
       </c>
       <c r="F47" s="5">
-        <v>1000</v>
+        <v>10419.959999999999</v>
       </c>
       <c r="G47" s="5">
         <f t="shared" si="0"/>
-        <v>5000</v>
+        <v>52099.799999999996</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B48" s="5">
-        <v>1191.96</v>
+        <v>1000</v>
       </c>
       <c r="C48" s="5">
-        <v>1191.96</v>
+        <v>1000</v>
       </c>
       <c r="D48" s="5">
-        <v>1191.96</v>
+        <v>1000</v>
       </c>
       <c r="E48" s="5">
-        <v>1191.96</v>
+        <v>1000</v>
       </c>
       <c r="F48" s="5">
-        <v>1191.96</v>
+        <v>1000</v>
       </c>
       <c r="G48" s="5">
         <f t="shared" si="0"/>
-        <v>5959.8</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B49" s="5">
-        <v>150000</v>
+        <v>1191.96</v>
       </c>
       <c r="C49" s="5">
-        <v>150000</v>
+        <v>1191.96</v>
       </c>
       <c r="D49" s="5">
-        <v>150000</v>
+        <v>1191.96</v>
       </c>
       <c r="E49" s="5">
-        <v>150000</v>
+        <v>1191.96</v>
       </c>
       <c r="F49" s="5">
-        <v>150000</v>
+        <v>1191.96</v>
       </c>
       <c r="G49" s="5">
         <f t="shared" si="0"/>
-        <v>750000</v>
+        <v>5959.8</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B50" s="5">
-        <v>5000</v>
+        <v>150000</v>
       </c>
       <c r="C50" s="5">
-        <v>5000</v>
+        <v>150000</v>
       </c>
       <c r="D50" s="5">
-        <v>5000</v>
+        <v>150000</v>
       </c>
       <c r="E50" s="5">
-        <v>5000</v>
+        <v>150000</v>
       </c>
       <c r="F50" s="5">
-        <v>5000</v>
+        <v>150000</v>
       </c>
       <c r="G50" s="5">
         <f t="shared" si="0"/>
-        <v>25000</v>
+        <v>750000</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B51" s="5">
-        <v>38160</v>
+        <v>5000</v>
       </c>
       <c r="C51" s="5">
-        <v>38160</v>
+        <v>5000</v>
       </c>
       <c r="D51" s="5">
-        <v>38160</v>
+        <v>5000</v>
       </c>
       <c r="E51" s="5">
-        <v>38160</v>
+        <v>5000</v>
       </c>
       <c r="F51" s="5">
-        <v>38160</v>
+        <v>5000</v>
       </c>
       <c r="G51" s="5">
         <f t="shared" si="0"/>
-        <v>190800</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B52" s="5">
-        <v>348</v>
+        <v>38160</v>
       </c>
       <c r="C52" s="5">
-        <v>348</v>
+        <v>38160</v>
       </c>
       <c r="D52" s="5">
-        <v>348</v>
+        <v>38160</v>
       </c>
       <c r="E52" s="5">
-        <v>348</v>
+        <v>38160</v>
       </c>
       <c r="F52" s="5">
-        <v>348</v>
+        <v>38160</v>
       </c>
       <c r="G52" s="5">
         <f t="shared" si="0"/>
-        <v>1740</v>
+        <v>190800</v>
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B53" s="5">
-        <v>1800</v>
+        <v>348</v>
       </c>
       <c r="C53" s="5">
-        <v>1800</v>
+        <v>348</v>
       </c>
       <c r="D53" s="5">
-        <v>1800</v>
+        <v>348</v>
       </c>
       <c r="E53" s="5">
-        <v>1800</v>
+        <v>348</v>
       </c>
       <c r="F53" s="5">
-        <v>1800</v>
+        <v>348</v>
       </c>
       <c r="G53" s="5">
         <f t="shared" si="0"/>
-        <v>9000</v>
+        <v>1740</v>
       </c>
     </row>
     <row r="54" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="B54" s="5">
-        <v>2500</v>
+        <v>1800</v>
       </c>
       <c r="C54" s="5">
-        <v>2500</v>
+        <v>1800</v>
       </c>
       <c r="D54" s="5">
-        <v>2500</v>
+        <v>1800</v>
       </c>
       <c r="E54" s="5">
-        <v>2500</v>
+        <v>1800</v>
       </c>
       <c r="F54" s="5">
-        <v>2500</v>
+        <v>1800</v>
       </c>
       <c r="G54" s="5">
         <f t="shared" si="0"/>
-        <v>12500</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="B55" s="5">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="C55" s="5">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="D55" s="5">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="E55" s="5">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="F55" s="5">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="G55" s="5">
         <f t="shared" si="0"/>
-        <v>15000</v>
+        <v>12500</v>
       </c>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B56" s="5">
-        <v>2400</v>
+        <v>3000</v>
       </c>
       <c r="C56" s="5">
-        <v>2400</v>
+        <v>3000</v>
       </c>
       <c r="D56" s="5">
-        <v>2400</v>
+        <v>3000</v>
       </c>
       <c r="E56" s="5">
-        <v>2400</v>
+        <v>3000</v>
       </c>
       <c r="F56" s="5">
-        <v>2400</v>
+        <v>3000</v>
       </c>
       <c r="G56" s="5">
         <f t="shared" si="0"/>
-        <v>12000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B57" s="5">
+        <v>2400</v>
+      </c>
+      <c r="C57" s="5">
+        <v>2400</v>
+      </c>
+      <c r="D57" s="5">
+        <v>2400</v>
+      </c>
+      <c r="E57" s="5">
+        <v>2400</v>
+      </c>
+      <c r="F57" s="5">
+        <v>2400</v>
+      </c>
+      <c r="G57" s="5">
+        <f t="shared" si="0"/>
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B58" s="5">
+        <v>240</v>
+      </c>
+      <c r="C58" s="5">
+        <v>240</v>
+      </c>
+      <c r="D58" s="5">
+        <v>240</v>
+      </c>
+      <c r="E58" s="5">
+        <v>240</v>
+      </c>
+      <c r="F58" s="5">
+        <v>240</v>
+      </c>
+      <c r="G58" s="5">
+        <f t="shared" si="0"/>
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A59" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B57" s="5">
-        <v>240</v>
-      </c>
-      <c r="C57" s="5">
-        <v>240</v>
-      </c>
-      <c r="D57" s="5">
-        <v>240</v>
-      </c>
-      <c r="E57" s="5">
-        <v>240</v>
-      </c>
-      <c r="F57" s="5">
-        <v>240</v>
-      </c>
-      <c r="G57" s="5">
-        <f t="shared" si="0"/>
-        <v>1200</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B58" s="7">
-        <f>SUM(B7:B57)</f>
+      <c r="B59" s="7">
+        <f>SUM(B8:B58)</f>
         <v>792001.91999999993</v>
       </c>
-      <c r="C58" s="7">
-        <f>SUM(C7:C57)</f>
+      <c r="C59" s="7">
+        <f>SUM(C8:C58)</f>
         <v>581322.92000000004</v>
       </c>
-      <c r="D58" s="7">
-        <f>SUM(D7:D57)</f>
+      <c r="D59" s="7">
+        <f>SUM(D8:D58)</f>
         <v>581322.92000000004</v>
       </c>
-      <c r="E58" s="7">
-        <f>SUM(E7:E57)</f>
+      <c r="E59" s="7">
+        <f>SUM(E8:E58)</f>
         <v>581322.92000000004</v>
       </c>
-      <c r="F58" s="7">
-        <f>SUM(F7:F57)</f>
+      <c r="F59" s="7">
+        <f>SUM(F8:F58)</f>
         <v>581322.92000000004</v>
       </c>
-      <c r="G58" s="10">
+      <c r="G59" s="10">
         <f t="shared" si="0"/>
         <v>3117293.5999999996</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="2"/>
-      <c r="B59" s="6"/>
-      <c r="C59" s="6"/>
-      <c r="D59" s="6"/>
-      <c r="E59" s="6"/>
-      <c r="F59" s="6"/>
-      <c r="G59" s="6"/>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A60" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="B60" s="5">
-        <f>B4 - B58</f>
-        <v>-345216.91999999993</v>
-      </c>
-      <c r="C60" s="5">
-        <f>C4 - C58</f>
-        <v>100926.07999999996</v>
-      </c>
-      <c r="D60" s="5">
-        <f>D4 - D58</f>
-        <v>245257.07999999996</v>
-      </c>
-      <c r="E60" s="5">
-        <f>E4 - E58</f>
-        <v>576188.07999999996</v>
-      </c>
-      <c r="F60" s="5">
-        <f>F4 - F58</f>
-        <v>881066.08</v>
-      </c>
-      <c r="G60" s="8">
-        <f>G4-G58</f>
-        <v>1458220.4000000004</v>
-      </c>
+    <row r="60" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="2"/>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6"/>
+      <c r="D60" s="6"/>
+      <c r="E60" s="6"/>
+      <c r="F60" s="6"/>
+      <c r="G60" s="6"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B61" s="5">
-        <f>IF(B60&gt;0,B60,0)</f>
-        <v>0</v>
+        <f>B4 - B59</f>
+        <v>-345216.91999999993</v>
       </c>
       <c r="C61" s="5">
-        <f>IF(C60&gt;0,C60,0)</f>
-        <v>100926.07999999996</v>
+        <f>C4 - C59</f>
+        <v>-22841.920000000042</v>
       </c>
       <c r="D61" s="5">
-        <f>IF(D60&gt;0,D60,0)</f>
-        <v>245257.07999999996</v>
+        <f>D4 - D59</f>
+        <v>116778.07999999996</v>
       </c>
       <c r="E61" s="5">
-        <f>IF(E60&gt;0,E60,0)</f>
-        <v>576188.07999999996</v>
+        <f>E4 - E59</f>
+        <v>291303.07999999996</v>
       </c>
       <c r="F61" s="5">
-        <f>IF(F60&gt;0,F60,0)</f>
-        <v>881066.08</v>
+        <f>F4 - F59</f>
+        <v>509460.07999999996</v>
       </c>
       <c r="G61" s="8">
-        <f>SUM(B61:F61)</f>
-        <v>1803437.3199999998</v>
+        <f>G4-G59</f>
+        <v>549482.40000000037</v>
       </c>
     </row>
     <row r="62" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B62" s="5">
-        <f>IF(B60&lt;0,B60,0)</f>
-        <v>-345216.91999999993</v>
+        <f>IF(B61&gt;0,B61,0)</f>
+        <v>0</v>
       </c>
       <c r="C62" s="5">
-        <f>IF(C60&lt;0,C60,0)</f>
+        <f>IF(C61&gt;0,C61,0)</f>
         <v>0</v>
       </c>
       <c r="D62" s="5">
-        <f>IF(D60&lt;0,D60,0)</f>
-        <v>0</v>
+        <f>IF(D61&gt;0,D61,0)</f>
+        <v>116778.07999999996</v>
       </c>
       <c r="E62" s="5">
-        <f>IF(E60&lt;0,E60,0)</f>
-        <v>0</v>
+        <f>IF(E61&gt;0,E61,0)</f>
+        <v>291303.07999999996</v>
       </c>
       <c r="F62" s="5">
-        <f>IF(F60&lt;0,F60,0)</f>
-        <v>0</v>
+        <f>IF(F61&gt;0,F61,0)</f>
+        <v>509460.07999999996</v>
       </c>
       <c r="G62" s="8">
         <f>SUM(B62:F62)</f>
-        <v>-345216.91999999993</v>
+        <v>917541.23999999987</v>
       </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B63" s="5">
-        <f>B60</f>
+        <f>IF(B61&lt;0,B61,0)</f>
         <v>-345216.91999999993</v>
       </c>
       <c r="C63" s="5">
-        <f>B63+C60</f>
-        <v>-244290.83999999997</v>
+        <f>IF(C61&lt;0,C61,0)</f>
+        <v>-22841.920000000042</v>
       </c>
       <c r="D63" s="5">
-        <f>C63+D60</f>
-        <v>966.23999999999069</v>
+        <f>IF(D61&lt;0,D61,0)</f>
+        <v>0</v>
       </c>
       <c r="E63" s="5">
-        <f>D63+E60</f>
-        <v>577154.31999999995</v>
+        <f>IF(E61&lt;0,E61,0)</f>
+        <v>0</v>
       </c>
       <c r="F63" s="5">
-        <f>E63+F60</f>
-        <v>1458220.4</v>
+        <f>IF(F61&lt;0,F61,0)</f>
+        <v>0</v>
       </c>
       <c r="G63" s="8">
         <f>SUM(B63:F63)</f>
-        <v>1446833.2</v>
+        <v>-368058.83999999997</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B64" s="5">
+        <f>B61</f>
+        <v>-345216.91999999993</v>
+      </c>
+      <c r="C64" s="5">
+        <f>B64+C61</f>
+        <v>-368058.83999999997</v>
+      </c>
+      <c r="D64" s="5">
+        <f>C64+D61</f>
+        <v>-251280.76</v>
+      </c>
+      <c r="E64" s="5">
+        <f>D64+E61</f>
+        <v>40022.319999999949</v>
+      </c>
+      <c r="F64" s="5">
+        <f>E64+F61</f>
+        <v>549482.39999999991</v>
+      </c>
+      <c r="G64" s="8">
+        <f>SUM(B64:F64)</f>
+        <v>-375051.80000000005</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B65" s="5">
+        <f>B61</f>
+        <v>-345216.91999999993</v>
+      </c>
+      <c r="C65" s="5">
+        <f>B65+C5-C59</f>
+        <v>-345718.83999999997</v>
+      </c>
+      <c r="D65" s="5">
+        <f>C65+D5-D59</f>
+        <v>-171974.76</v>
+      </c>
+      <c r="E65" s="5">
+        <f>D65+E5-E59</f>
+        <v>228289.31999999995</v>
+      </c>
+      <c r="F65" s="5">
+        <f>E65+F5-F59</f>
+        <v>923029.39999999979</v>
+      </c>
+      <c r="G65" s="8">
+        <f>SUM(B65:F65)</f>
+        <v>288408.19999999984</v>
       </c>
     </row>
   </sheetData>

</xml_diff>